<commit_message>
Update from CPU test run
</commit_message>
<xml_diff>
--- a/phys5v48hw/hw6/hw6CPUData.xlsx
+++ b/phys5v48hw/hw6/hw6CPUData.xlsx
@@ -439,7 +439,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>0.0015572579577565193</t>
+          <t>0.002077734097838402</t>
         </is>
       </c>
     </row>
@@ -454,7 +454,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>9.390106424689293e-05</t>
+          <t>0.0003140460466966033</t>
         </is>
       </c>
     </row>
@@ -469,7 +469,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>2.4950015358626842e-05</t>
+          <t>8.161808364093304e-05</t>
         </is>
       </c>
     </row>

</xml_diff>